<commit_message>
Completar atualização de loterias - preencher gaps de concursos faltantes até 21/08/2026
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/dia_sorte_asloterias_ate_concurso_1242_crescente.xlsx
+++ b/historicoresultadosloteriasnacionais/dia_sorte_asloterias_ate_concurso_1242_crescente.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1273"/>
+  <dimension ref="A1:J1286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,6 @@
       <c r="I1" t="n">
         <v>30</v>
       </c>
-      <c r="J1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -478,7 +477,6 @@
       <c r="I2" t="n">
         <v>22</v>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -510,7 +508,6 @@
       <c r="I3" t="n">
         <v>17</v>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -542,7 +539,6 @@
       <c r="I4" t="n">
         <v>29</v>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -574,7 +570,6 @@
       <c r="I5" t="n">
         <v>29</v>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -606,7 +601,6 @@
       <c r="I6" t="n">
         <v>31</v>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -638,7 +632,6 @@
       <c r="I7" t="n">
         <v>31</v>
       </c>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -670,7 +663,6 @@
       <c r="I8" t="n">
         <v>30</v>
       </c>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -702,7 +694,6 @@
       <c r="I9" t="n">
         <v>22</v>
       </c>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -734,7 +725,6 @@
       <c r="I10" t="n">
         <v>26</v>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -766,7 +756,6 @@
       <c r="I11" t="n">
         <v>28</v>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -798,7 +787,6 @@
       <c r="I12" t="n">
         <v>30</v>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -830,7 +818,6 @@
       <c r="I13" t="n">
         <v>28</v>
       </c>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -862,7 +849,6 @@
       <c r="I14" t="n">
         <v>27</v>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -894,7 +880,6 @@
       <c r="I15" t="n">
         <v>28</v>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -926,7 +911,6 @@
       <c r="I16" t="n">
         <v>28</v>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -958,7 +942,6 @@
       <c r="I17" t="n">
         <v>28</v>
       </c>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -990,7 +973,6 @@
       <c r="I18" t="n">
         <v>25</v>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1022,7 +1004,6 @@
       <c r="I19" t="n">
         <v>31</v>
       </c>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1054,7 +1035,6 @@
       <c r="I20" t="n">
         <v>31</v>
       </c>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1086,7 +1066,6 @@
       <c r="I21" t="n">
         <v>18</v>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1118,7 +1097,6 @@
       <c r="I22" t="n">
         <v>26</v>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1150,7 +1128,6 @@
       <c r="I23" t="n">
         <v>25</v>
       </c>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1161,14 +1138,6 @@
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1176,15 +1145,6 @@
           <t>As Loterias - www.asloterias.com.br - Todos Resultados da Dia de Sorte</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1192,15 +1152,6 @@
           <t>Este arquivo foi baixado no site www.asloterias.com.br no dia 11/07/2026</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1208,56 +1159,16 @@
           <t>Visite o site para baixar a versão mais atualizada deste arquivo!</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
           <t>TODOS RESULTADOS DA DIA DE SORTE</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
@@ -34748,7 +34659,6 @@
       <c r="I960" t="n">
         <v>26</v>
       </c>
-      <c r="J960" t="inlineStr"/>
     </row>
     <row r="961">
       <c r="A961" t="n">
@@ -46015,6 +45925,526 @@
       <c r="J1273" t="inlineStr">
         <is>
           <t>Fevereiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="n">
+        <v>1266</v>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G1274" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I1274" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="n">
+        <v>1267</v>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G1275" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="I1275" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="n">
+        <v>1268</v>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="G1276" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="I1276" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="n">
+        <v>1269</v>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="G1277" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="I1277" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="n">
+        <v>1270</v>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G1278" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="I1278" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="n">
+        <v>1271</v>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="G1279" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="I1279" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G1280" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I1280" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="n">
+        <v>1277</v>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G1281" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="I1281" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G1282" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="I1282" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="n">
+        <v>1273</v>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G1283" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="I1283" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="n">
+        <v>1274</v>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G1284" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="I1284" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="n">
+        <v>1275</v>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="G1285" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="I1285" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="n">
+        <v>1276</v>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="G1286" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="I1286" t="inlineStr">
+        <is>
+          <t>28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrigir datas dos concursos que estavam com nan - usar dataApuracao da API e converter formato
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/dia_sorte_asloterias_ate_concurso_1242_crescente.xlsx
+++ b/historicoresultadosloteriasnacionais/dia_sorte_asloterias_ate_concurso_1242_crescente.xlsx
@@ -45932,6 +45932,11 @@
       <c r="A1274" t="n">
         <v>1266</v>
       </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
       <c r="C1274" t="inlineStr">
         <is>
           <t>04</t>
@@ -45972,6 +45977,11 @@
       <c r="A1275" t="n">
         <v>1267</v>
       </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="C1275" t="inlineStr">
         <is>
           <t>02</t>
@@ -46012,6 +46022,11 @@
       <c r="A1276" t="n">
         <v>1268</v>
       </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="C1276" t="inlineStr">
         <is>
           <t>08</t>
@@ -46052,6 +46067,11 @@
       <c r="A1277" t="n">
         <v>1269</v>
       </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
       <c r="C1277" t="inlineStr">
         <is>
           <t>06</t>
@@ -46092,6 +46112,11 @@
       <c r="A1278" t="n">
         <v>1270</v>
       </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="C1278" t="inlineStr">
         <is>
           <t>06</t>
@@ -46132,6 +46157,11 @@
       <c r="A1279" t="n">
         <v>1271</v>
       </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="C1279" t="inlineStr">
         <is>
           <t>05</t>
@@ -46172,6 +46202,11 @@
       <c r="A1280" t="n">
         <v>1272</v>
       </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
       <c r="C1280" t="inlineStr">
         <is>
           <t>01</t>
@@ -46212,6 +46247,11 @@
       <c r="A1281" t="n">
         <v>1277</v>
       </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
       <c r="C1281" t="inlineStr">
         <is>
           <t>01</t>
@@ -46252,6 +46292,11 @@
       <c r="A1282" t="n">
         <v>1278</v>
       </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
       <c r="C1282" t="inlineStr">
         <is>
           <t>01</t>
@@ -46292,6 +46337,11 @@
       <c r="A1283" t="n">
         <v>1273</v>
       </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
       <c r="C1283" t="inlineStr">
         <is>
           <t>07</t>
@@ -46332,6 +46382,11 @@
       <c r="A1284" t="n">
         <v>1274</v>
       </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
       <c r="C1284" t="inlineStr">
         <is>
           <t>08</t>
@@ -46372,6 +46427,11 @@
       <c r="A1285" t="n">
         <v>1275</v>
       </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
       <c r="C1285" t="inlineStr">
         <is>
           <t>05</t>
@@ -46411,6 +46471,11 @@
     <row r="1286">
       <c r="A1286" t="n">
         <v>1276</v>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
       </c>
       <c r="C1286" t="inlineStr">
         <is>

</xml_diff>